<commit_message>
dataset ETF: aggiunto IWMO.MI (World Momentum Factor)
Quarantadue ticker invece di quarantuno. Il titolo era stato aggiunto al
Foglio21 di portafoglio/ETF.xlsx, che e' il foglio di lavoro e non lo legge
nessuno: i dataset condivisi li prende Files/*.xlsx (_FILES_DIR in
portafoglio, _FE_FILES_DIR in frontiera, e i job notturni ciclano su quello).

Sta fra IVE e ZPRV.DE come nel foglio di lavoro, cosi' il blocco degli
azionari USA resta insieme. La valuta e' EUR, non "ERR" come nel foglio:
IWMO.MI quota a Milano in euro, e comunque comanda quella di Yahoo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portafoglio/ETF.xlsx
+++ b/portafoglio/ETF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Downloads/andcappe_zip/Dashboard/SITO_WEB/Sito personale/portafoglio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BC11CF7-0E93-5940-A76B-7711893FA9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5C71231-3FB7-7F4F-94E0-3760C2344279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4380" yWindow="0" windowWidth="24420" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7586" uniqueCount="2756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7590" uniqueCount="2759">
   <si>
     <t>Simbolo</t>
   </si>
@@ -8579,6 +8579,15 @@
   </si>
   <si>
     <t>Bench AZ. VANGUARD ACWI</t>
+  </si>
+  <si>
+    <t>Az. World Momentum Factor</t>
+  </si>
+  <si>
+    <t>ERR</t>
+  </si>
+  <si>
+    <t>Azionari World Momentum Factor</t>
   </si>
 </sst>
 </file>
@@ -9889,16 +9898,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="101" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="85" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="82" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="102" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -9915,6 +9914,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="105" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="85" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="82" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -9923,91 +9932,6 @@
     <cellStyle name="Percentuale" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -10108,6 +10032,91 @@
         <name val="Helvetica Neue"/>
         <family val="2"/>
         <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
       </font>
     </dxf>
     <dxf>
@@ -15599,6 +15608,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -15606,7 +15616,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -16304,26 +16313,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D30" totalsRowShown="0" headerRowDxfId="11" dataDxfId="0">
-  <autoFilter ref="A1:D30" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D31" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:D31" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{036B7D95-54D0-CE4A-A97C-6EC741E876E4}" name="VALUTA" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{BC856CD8-BE7C-D246-AFFE-8A0458341DA0}" name="CLASSE" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{D2DEAFE7-7181-F841-96D9-E16F6CD58118}" name="DESCRIZIONE" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{036B7D95-54D0-CE4A-A97C-6EC741E876E4}" name="VALUTA" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{BC856CD8-BE7C-D246-AFFE-8A0458341DA0}" name="CLASSE" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}" name="Tabella323" displayName="Tabella323" ref="A1:D53" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}" name="Tabella323" displayName="Tabella323" ref="A1:D53" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="A1:D53" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{99BE53A6-82BE-7C4C-8EDB-FC2585DE7E29}" name="SIMBOLO" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{79CB9D70-57D7-004E-8DD2-11CA0A269F24}" name="DESCRIZIONE" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{4221CAB4-B4C0-5746-BDF4-C3FC111D5F78}" name="VALUTA" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{530400BE-E6AA-4A47-B046-BF29D0205198}" name="CLASSE" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{99BE53A6-82BE-7C4C-8EDB-FC2585DE7E29}" name="SIMBOLO" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{79CB9D70-57D7-004E-8DD2-11CA0A269F24}" name="DESCRIZIONE" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{4221CAB4-B4C0-5746-BDF4-C3FC111D5F78}" name="VALUTA" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{530400BE-E6AA-4A47-B046-BF29D0205198}" name="CLASSE" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17434,7 +17443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C714FF38-E71E-3648-9A7A-13401C8B9393}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11"/>
   <cols>
     <col min="1" max="1" width="11.83203125" style="233" customWidth="1"/>
@@ -17457,422 +17466,436 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="12">
-      <c r="A2" s="238" t="s">
+      <c r="A2" s="234" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="239" t="s">
+      <c r="B2" s="235" t="s">
         <v>2755</v>
       </c>
-      <c r="C2" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="240" t="s">
+      <c r="C2" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="236" t="s">
         <v>2747</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="12">
-      <c r="A3" s="241" t="s">
+      <c r="A3" s="237" t="s">
         <v>2571</v>
       </c>
-      <c r="B3" s="241" t="s">
+      <c r="B3" s="237" t="s">
         <v>2751</v>
       </c>
-      <c r="C3" s="242" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="243" t="s">
+      <c r="C3" s="238" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="239" t="s">
         <v>2723</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12">
-      <c r="A4" s="240" t="s">
+      <c r="A4" s="236" t="s">
         <v>2255</v>
       </c>
-      <c r="B4" s="241" t="s">
+      <c r="B4" s="237" t="s">
         <v>2753</v>
       </c>
-      <c r="C4" s="244" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="243" t="s">
+      <c r="C4" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="239" t="s">
         <v>2723</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="12">
-      <c r="A5" s="241" t="s">
+      <c r="A5" s="237" t="s">
         <v>2750</v>
       </c>
-      <c r="B5" s="241" t="s">
+      <c r="B5" s="237" t="s">
         <v>2754</v>
       </c>
-      <c r="C5" s="244" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="243" t="s">
+      <c r="C5" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="239" t="s">
         <v>2723</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12">
-      <c r="A6" s="240" t="s">
+      <c r="A6" s="236" t="s">
         <v>2617</v>
       </c>
-      <c r="B6" s="241" t="s">
+      <c r="B6" s="237" t="s">
         <v>2752</v>
       </c>
-      <c r="C6" s="244" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="243" t="s">
+      <c r="C6" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="239" t="s">
         <v>2723</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="12">
-      <c r="A7" s="238" t="s">
+      <c r="A7" s="234" t="s">
         <v>2619</v>
       </c>
-      <c r="B7" s="241" t="s">
+      <c r="B7" s="237" t="s">
         <v>2724</v>
       </c>
-      <c r="C7" s="240" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="240" t="s">
+      <c r="C7" s="236" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="236" t="s">
         <v>2696</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="12">
-      <c r="A8" s="240" t="s">
+      <c r="A8" s="236" t="s">
         <v>1091</v>
       </c>
-      <c r="B8" s="241" t="s">
+      <c r="B8" s="237" t="s">
         <v>2734</v>
       </c>
-      <c r="C8" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="240" t="s">
+      <c r="C8" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="236" t="s">
         <v>2635</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="12">
-      <c r="A9" s="240" t="s">
+      <c r="A9" s="236" t="s">
         <v>2706</v>
       </c>
-      <c r="B9" s="241" t="s">
+      <c r="B9" s="237" t="s">
         <v>2731</v>
       </c>
-      <c r="C9" s="240" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="240" t="s">
+      <c r="C9" s="236" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="236" t="s">
         <v>2708</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="12">
-      <c r="A10" s="240" t="s">
+      <c r="A10" s="236" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="240" t="s">
+      <c r="B10" s="236" t="s">
         <v>2748</v>
       </c>
-      <c r="C10" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="240" t="s">
+      <c r="C10" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="236" t="s">
         <v>2749</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="12">
-      <c r="A11" s="240" t="s">
+      <c r="A11" s="236" t="s">
         <v>2668</v>
       </c>
-      <c r="B11" s="240" t="s">
+      <c r="B11" s="236" t="s">
         <v>2725</v>
       </c>
-      <c r="C11" s="240" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="240" t="s">
+      <c r="C11" s="236" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="236" t="s">
         <v>2673</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="12">
-      <c r="A12" s="240" t="s">
+      <c r="A12" s="236" t="s">
         <v>1089</v>
       </c>
-      <c r="B12" s="240" t="s">
+      <c r="B12" s="236" t="s">
         <v>2726</v>
       </c>
-      <c r="C12" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="240" t="s">
+      <c r="C12" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="236" t="s">
         <v>2680</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="12">
-      <c r="A13" s="245" t="s">
+      <c r="A13" s="241" t="s">
         <v>2704</v>
       </c>
-      <c r="B13" s="240" t="s">
+      <c r="B13" s="236" t="s">
         <v>2727</v>
       </c>
-      <c r="C13" s="240" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="240" t="s">
+      <c r="C13" s="236" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="236" t="s">
         <v>2685</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="12">
-      <c r="A14" s="240" t="s">
+      <c r="A14" s="236" t="s">
         <v>2681</v>
       </c>
-      <c r="B14" s="240" t="s">
+      <c r="B14" s="236" t="s">
         <v>2728</v>
       </c>
-      <c r="C14" s="240" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="240" t="s">
+      <c r="C14" s="236" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="236" t="s">
         <v>2686</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="12">
-      <c r="A15" s="240" t="s">
+      <c r="A15" s="236" t="s">
         <v>2683</v>
       </c>
-      <c r="B15" s="240" t="s">
+      <c r="B15" s="236" t="s">
         <v>2729</v>
       </c>
-      <c r="C15" s="240" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="240" t="s">
+      <c r="C15" s="236" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="236" t="s">
         <v>2687</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="12">
-      <c r="A16" s="245" t="s">
+      <c r="A16" s="236" t="s">
+        <v>1744</v>
+      </c>
+      <c r="B16" s="236" t="s">
+        <v>2756</v>
+      </c>
+      <c r="C16" s="236" t="s">
+        <v>2757</v>
+      </c>
+      <c r="D16" s="236" t="s">
+        <v>2758</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="12">
+      <c r="A17" s="241" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="240" t="s">
+      <c r="B17" s="236" t="s">
         <v>2730</v>
       </c>
-      <c r="C16" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="240" t="s">
+      <c r="C17" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="236" t="s">
         <v>2691</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="12">
-      <c r="A17" s="240" t="s">
+    <row r="18" spans="1:4" ht="12">
+      <c r="A18" s="236" t="s">
         <v>1872</v>
       </c>
-      <c r="B17" s="240" t="s">
+      <c r="B18" s="236" t="s">
         <v>2733</v>
       </c>
-      <c r="C17" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="240" t="s">
+      <c r="C18" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="236" t="s">
         <v>2694</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="12">
-      <c r="A18" s="240" t="s">
+    <row r="19" spans="1:4" ht="12">
+      <c r="A19" s="236" t="s">
         <v>833</v>
       </c>
-      <c r="B18" s="240" t="s">
+      <c r="B19" s="236" t="s">
         <v>2732</v>
       </c>
-      <c r="C18" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="240" t="s">
+      <c r="C19" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="236" t="s">
         <v>2692</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="12">
-      <c r="A19" s="240" t="s">
+    <row r="20" spans="1:4" ht="12">
+      <c r="A20" s="236" t="s">
         <v>2636</v>
       </c>
-      <c r="B19" s="240" t="s">
+      <c r="B20" s="236" t="s">
         <v>2735</v>
       </c>
-      <c r="C19" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="240" t="s">
+      <c r="C20" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="236" t="s">
         <v>2640</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="12">
-      <c r="A20" s="240" t="s">
+    <row r="21" spans="1:4" ht="12">
+      <c r="A21" s="236" t="s">
         <v>1090</v>
       </c>
-      <c r="B20" s="240" t="s">
+      <c r="B21" s="236" t="s">
         <v>2736</v>
       </c>
-      <c r="C20" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="240" t="s">
+      <c r="C21" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="236" t="s">
         <v>2644</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="12">
-      <c r="A21" s="245" t="s">
+    <row r="22" spans="1:4" ht="12">
+      <c r="A22" s="241" t="s">
         <v>2720</v>
       </c>
-      <c r="B21" s="245" t="s">
+      <c r="B22" s="241" t="s">
         <v>2737</v>
       </c>
-      <c r="C21" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="240" t="s">
+      <c r="C22" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="236" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="12">
-      <c r="A22" s="245" t="s">
+    <row r="23" spans="1:4" ht="12">
+      <c r="A23" s="241" t="s">
         <v>2177</v>
       </c>
-      <c r="B22" s="245" t="s">
+      <c r="B23" s="241" t="s">
         <v>2738</v>
       </c>
-      <c r="C22" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="240" t="s">
+      <c r="C23" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="236" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="12">
-      <c r="A23" s="245" t="s">
+    <row r="24" spans="1:4" ht="12">
+      <c r="A24" s="241" t="s">
         <v>2721</v>
       </c>
-      <c r="B23" s="245" t="s">
+      <c r="B24" s="241" t="s">
         <v>2739</v>
       </c>
-      <c r="C23" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="240" t="s">
+      <c r="C24" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="236" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="12">
-      <c r="A24" s="240" t="s">
+    <row r="25" spans="1:4" ht="12">
+      <c r="A25" s="236" t="s">
         <v>2656</v>
       </c>
-      <c r="B24" s="240" t="s">
+      <c r="B25" s="236" t="s">
         <v>2740</v>
       </c>
-      <c r="C24" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" s="240" t="s">
+      <c r="C25" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="236" t="s">
         <v>2660</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="12">
-      <c r="A25" s="240" t="s">
+    <row r="26" spans="1:4" ht="12">
+      <c r="A26" s="236" t="s">
         <v>2710</v>
       </c>
-      <c r="B25" s="241" t="s">
+      <c r="B26" s="237" t="s">
         <v>2741</v>
       </c>
-      <c r="C25" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="240" t="s">
+      <c r="C26" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="236" t="s">
         <v>2660</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="12">
-      <c r="A26" s="240" t="s">
+    <row r="27" spans="1:4" ht="12">
+      <c r="A27" s="236" t="s">
         <v>2712</v>
       </c>
-      <c r="B26" s="241" t="s">
+      <c r="B27" s="237" t="s">
         <v>2742</v>
       </c>
-      <c r="C26" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="240" t="s">
+      <c r="C27" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="236" t="s">
         <v>2662</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="12">
-      <c r="A27" s="245" t="s">
+    <row r="28" spans="1:4" ht="12">
+      <c r="A28" s="241" t="s">
         <v>2663</v>
       </c>
-      <c r="B27" s="240" t="s">
+      <c r="B28" s="236" t="s">
         <v>2743</v>
       </c>
-      <c r="C27" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" s="240" t="s">
+      <c r="C28" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="236" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="12">
-      <c r="A28" s="245" t="s">
+    <row r="29" spans="1:4" ht="12">
+      <c r="A29" s="241" t="s">
         <v>2722</v>
       </c>
-      <c r="B28" s="245" t="s">
+      <c r="B29" s="241" t="s">
         <v>2744</v>
       </c>
-      <c r="C28" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D28" s="240" t="s">
+      <c r="C29" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="236" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="12">
-      <c r="A29" s="240" t="s">
+    <row r="30" spans="1:4" ht="12">
+      <c r="A30" s="236" t="s">
         <v>2718</v>
       </c>
-      <c r="B29" s="241" t="s">
+      <c r="B30" s="237" t="s">
         <v>2745</v>
       </c>
-      <c r="C29" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D29" s="240" t="s">
+      <c r="C30" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="236" t="s">
         <v>2667</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="12">
-      <c r="A30" s="240" t="s">
+    <row r="31" spans="1:4" ht="12">
+      <c r="A31" s="236" t="s">
         <v>2697</v>
       </c>
-      <c r="B30" s="240" t="s">
+      <c r="B31" s="236" t="s">
         <v>2746</v>
       </c>
-      <c r="C30" s="240" t="s">
-        <v>28</v>
-      </c>
-      <c r="D30" s="240" t="s">
+      <c r="C31" s="236" t="s">
+        <v>28</v>
+      </c>
+      <c r="D31" s="236" t="s">
         <v>2089</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="95" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="A27" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
-    <hyperlink ref="A16" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
+    <hyperlink ref="A28" r:id="rId1" display="http://xgin.de/" xr:uid="{6D042F4B-B1B6-714D-834A-FF03BB9AF65F}"/>
+    <hyperlink ref="A17" r:id="rId2" display="http://zprv.de/" xr:uid="{AE8F80AC-32A6-C643-BEE6-694ECBB145F6}"/>
     <hyperlink ref="A13" r:id="rId3" display="http://iusg.de/" xr:uid="{C28C7857-119A-4744-B0BB-4DDEA3E95E35}"/>
-    <hyperlink ref="B21" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
-    <hyperlink ref="B22" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
-    <hyperlink ref="B23" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
-    <hyperlink ref="A28" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
-    <hyperlink ref="B28" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
+    <hyperlink ref="B22" r:id="rId4" display="https://finance.yahoo.com/quote/CSBGE3.MI/" xr:uid="{07F4F9CA-E0FA-1C49-87F4-4EBCF7177C7D}"/>
+    <hyperlink ref="B23" r:id="rId5" display="https://finance.yahoo.com/quote/CSBGE7.MI/" xr:uid="{02FC7EA0-25C6-E34E-AB6A-3622B551A50D}"/>
+    <hyperlink ref="B24" r:id="rId6" display="https://finance.yahoo.com/quote/SXRQ.DE/" xr:uid="{4E4D2C26-5E71-C644-AF09-EF7691622628}"/>
+    <hyperlink ref="A29" r:id="rId7" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{6DA783E3-A09C-7C47-88D8-23C14B21E7FE}"/>
+    <hyperlink ref="B29" r:id="rId8" display="https://finance.yahoo.com/quote/XEIN.DE/" xr:uid="{894A731F-3358-3D4B-A900-50AD652ED5AE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -17892,20 +17915,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17">
-      <c r="A1" s="236" t="s">
+      <c r="A1" s="244" t="s">
         <v>2346</v>
       </c>
-      <c r="B1" s="235"/>
-      <c r="C1" s="235"/>
-      <c r="D1" s="235"/>
+      <c r="B1" s="243"/>
+      <c r="C1" s="243"/>
+      <c r="D1" s="243"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="237" t="s">
+      <c r="A2" s="245" t="s">
         <v>2347</v>
       </c>
-      <c r="B2" s="235"/>
-      <c r="C2" s="235"/>
-      <c r="D2" s="235"/>
+      <c r="B2" s="243"/>
+      <c r="C2" s="243"/>
+      <c r="D2" s="243"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="181" t="s">
@@ -17922,12 +17945,12 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="234" t="s">
+      <c r="A4" s="242" t="s">
         <v>2349</v>
       </c>
-      <c r="B4" s="235"/>
-      <c r="C4" s="235"/>
-      <c r="D4" s="235"/>
+      <c r="B4" s="243"/>
+      <c r="C4" s="243"/>
+      <c r="D4" s="243"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="182" t="s">
@@ -18154,12 +18177,12 @@
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="234" t="s">
+      <c r="A21" s="242" t="s">
         <v>2377</v>
       </c>
-      <c r="B21" s="235"/>
-      <c r="C21" s="235"/>
-      <c r="D21" s="235"/>
+      <c r="B21" s="243"/>
+      <c r="C21" s="243"/>
+      <c r="D21" s="243"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="186" t="s">
@@ -18204,12 +18227,12 @@
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="234" t="s">
+      <c r="A25" s="242" t="s">
         <v>2384</v>
       </c>
-      <c r="B25" s="235"/>
-      <c r="C25" s="235"/>
-      <c r="D25" s="235"/>
+      <c r="B25" s="243"/>
+      <c r="C25" s="243"/>
+      <c r="D25" s="243"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="186" t="s">
@@ -18254,12 +18277,12 @@
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="234" t="s">
+      <c r="A29" s="242" t="s">
         <v>2391</v>
       </c>
-      <c r="B29" s="235"/>
-      <c r="C29" s="235"/>
-      <c r="D29" s="235"/>
+      <c r="B29" s="243"/>
+      <c r="C29" s="243"/>
+      <c r="D29" s="243"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="186" t="s">
@@ -18304,12 +18327,12 @@
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="234" t="s">
+      <c r="A33" s="242" t="s">
         <v>2395</v>
       </c>
-      <c r="B33" s="235"/>
-      <c r="C33" s="235"/>
-      <c r="D33" s="235"/>
+      <c r="B33" s="243"/>
+      <c r="C33" s="243"/>
+      <c r="D33" s="243"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="186" t="s">
@@ -18368,12 +18391,12 @@
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="234" t="s">
+      <c r="A38" s="242" t="s">
         <v>2403</v>
       </c>
-      <c r="B38" s="235"/>
-      <c r="C38" s="235"/>
-      <c r="D38" s="235"/>
+      <c r="B38" s="243"/>
+      <c r="C38" s="243"/>
+      <c r="D38" s="243"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="190" t="s">
@@ -18418,12 +18441,12 @@
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="234" t="s">
+      <c r="A42" s="242" t="s">
         <v>2410</v>
       </c>
-      <c r="B42" s="235"/>
-      <c r="C42" s="235"/>
-      <c r="D42" s="235"/>
+      <c r="B42" s="243"/>
+      <c r="C42" s="243"/>
+      <c r="D42" s="243"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="190" t="s">
@@ -18468,12 +18491,12 @@
       </c>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" s="234" t="s">
+      <c r="A46" s="242" t="s">
         <v>2417</v>
       </c>
-      <c r="B46" s="235"/>
-      <c r="C46" s="235"/>
-      <c r="D46" s="235"/>
+      <c r="B46" s="243"/>
+      <c r="C46" s="243"/>
+      <c r="D46" s="243"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="190" t="s">
@@ -18518,12 +18541,12 @@
       </c>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="234" t="s">
+      <c r="A50" s="242" t="s">
         <v>2424</v>
       </c>
-      <c r="B50" s="235"/>
-      <c r="C50" s="235"/>
-      <c r="D50" s="235"/>
+      <c r="B50" s="243"/>
+      <c r="C50" s="243"/>
+      <c r="D50" s="243"/>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="190" t="s">
@@ -18568,12 +18591,12 @@
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="234" t="s">
+      <c r="A54" s="242" t="s">
         <v>2431</v>
       </c>
-      <c r="B54" s="235"/>
-      <c r="C54" s="235"/>
-      <c r="D54" s="235"/>
+      <c r="B54" s="243"/>
+      <c r="C54" s="243"/>
+      <c r="D54" s="243"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="190" t="s">
@@ -18618,12 +18641,12 @@
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="234" t="s">
+      <c r="A58" s="242" t="s">
         <v>2437</v>
       </c>
-      <c r="B58" s="235"/>
-      <c r="C58" s="235"/>
-      <c r="D58" s="235"/>
+      <c r="B58" s="243"/>
+      <c r="C58" s="243"/>
+      <c r="D58" s="243"/>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="190" t="s">
@@ -18668,12 +18691,12 @@
       </c>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="234" t="s">
+      <c r="A62" s="242" t="s">
         <v>2444</v>
       </c>
-      <c r="B62" s="235"/>
-      <c r="C62" s="235"/>
-      <c r="D62" s="235"/>
+      <c r="B62" s="243"/>
+      <c r="C62" s="243"/>
+      <c r="D62" s="243"/>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="190" t="s">
@@ -18704,12 +18727,12 @@
       </c>
     </row>
     <row r="65" spans="1:4">
-      <c r="A65" s="234" t="s">
+      <c r="A65" s="242" t="s">
         <v>2449</v>
       </c>
-      <c r="B65" s="235"/>
-      <c r="C65" s="235"/>
-      <c r="D65" s="235"/>
+      <c r="B65" s="243"/>
+      <c r="C65" s="243"/>
+      <c r="D65" s="243"/>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="186" t="s">
@@ -18754,12 +18777,12 @@
       </c>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" s="234" t="s">
+      <c r="A69" s="242" t="s">
         <v>2455</v>
       </c>
-      <c r="B69" s="235"/>
-      <c r="C69" s="235"/>
-      <c r="D69" s="235"/>
+      <c r="B69" s="243"/>
+      <c r="C69" s="243"/>
+      <c r="D69" s="243"/>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="186" t="s">
@@ -18790,12 +18813,12 @@
       </c>
     </row>
     <row r="72" spans="1:4">
-      <c r="A72" s="234" t="s">
+      <c r="A72" s="242" t="s">
         <v>2460</v>
       </c>
-      <c r="B72" s="235"/>
-      <c r="C72" s="235"/>
-      <c r="D72" s="235"/>
+      <c r="B72" s="243"/>
+      <c r="C72" s="243"/>
+      <c r="D72" s="243"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="190" t="s">
@@ -18840,12 +18863,12 @@
       </c>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" s="234" t="s">
+      <c r="A76" s="242" t="s">
         <v>2467</v>
       </c>
-      <c r="B76" s="235"/>
-      <c r="C76" s="235"/>
-      <c r="D76" s="235"/>
+      <c r="B76" s="243"/>
+      <c r="C76" s="243"/>
+      <c r="D76" s="243"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="190" t="s">
@@ -18890,12 +18913,12 @@
       </c>
     </row>
     <row r="80" spans="1:4">
-      <c r="A80" s="234" t="s">
+      <c r="A80" s="242" t="s">
         <v>2474</v>
       </c>
-      <c r="B80" s="235"/>
-      <c r="C80" s="235"/>
-      <c r="D80" s="235"/>
+      <c r="B80" s="243"/>
+      <c r="C80" s="243"/>
+      <c r="D80" s="243"/>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="190" t="s">
@@ -18941,6 +18964,13 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A76:D76"/>
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -18953,13 +18983,6 @@
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A76:D76"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>